<commit_message>
ABP QA regression fixes
</commit_message>
<xml_diff>
--- a/KatalonData/ABPTestData/ABPTestData.xlsx
+++ b/KatalonData/ABPTestData/ABPTestData.xlsx
@@ -55,7 +55,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="336" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="346" uniqueCount="101">
   <si>
     <t>BillType</t>
   </si>
@@ -439,6 +439,21 @@
   </si>
   <si>
     <t>Fri Sep 18 01:02:30 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Sep 22 20:59:23 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Sep 22 23:37:32 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Sep 22 23:38:57 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Sep 22 23:40:26 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Sep 22 23:41:47 IST 2026</t>
   </si>
 </sst>
 </file>
@@ -1357,10 +1372,10 @@
     </row>
     <row r="2" spans="1:11" ht="362.5" x14ac:dyDescent="0.35">
       <c r="A2" t="s" s="0">
-        <v>55</v>
+        <v>34</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12" t="s">
@@ -1453,7 +1468,7 @@
         <v>34</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12" t="s">
@@ -1549,7 +1564,7 @@
         <v>34</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12" t="s">
@@ -1681,10 +1696,10 @@
     </row>
     <row r="2" spans="1:7" ht="246.5" x14ac:dyDescent="0.35">
       <c r="A2" t="s" s="0">
-        <v>55</v>
+        <v>34</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12" t="s">
@@ -1888,10 +1903,10 @@
     </row>
     <row r="2" spans="1:10" ht="232" x14ac:dyDescent="0.35">
       <c r="A2" t="s" s="0">
-        <v>55</v>
+        <v>34</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12" t="s">

</xml_diff>